<commit_message>
cambios menores en la app
</commit_message>
<xml_diff>
--- a/Pruebas/Rendimiento/Pruebas de rendimiento.xlsx
+++ b/Pruebas/Rendimiento/Pruebas de rendimiento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yagon\Desktop\Clase\Quinto año\TFG\Aplicacion\Pruebas\Rendimiento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169D8029-2559-4D30-9F25-F447181A14CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF68BF50-87A4-49A3-AE89-1C6778D0D214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tiempos" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="21">
   <si>
     <t>Descarga de datos</t>
   </si>
@@ -196,12 +196,14 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:M7"/>
+  <dimension ref="B2:Q7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5546875" customWidth="1"/>
@@ -491,78 +493,90 @@
     <col min="3" max="3" width="20.6640625" customWidth="1"/>
     <col min="4" max="4" width="17.88671875" customWidth="1"/>
     <col min="5" max="5" width="18.88671875" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="31.5546875" customWidth="1"/>
-    <col min="8" max="8" width="20.6640625" customWidth="1"/>
-    <col min="9" max="9" width="21.88671875" customWidth="1"/>
-    <col min="10" max="10" width="19.21875" customWidth="1"/>
-    <col min="11" max="11" width="19.33203125" customWidth="1"/>
-    <col min="12" max="12" width="20.21875" customWidth="1"/>
-    <col min="13" max="13" width="30.21875" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="31.5546875" customWidth="1"/>
+    <col min="9" max="9" width="14.77734375" customWidth="1"/>
+    <col min="10" max="10" width="20.6640625" customWidth="1"/>
+    <col min="11" max="11" width="21.88671875" customWidth="1"/>
+    <col min="12" max="12" width="19.21875" customWidth="1"/>
+    <col min="13" max="13" width="14.77734375" customWidth="1"/>
+    <col min="14" max="14" width="21" customWidth="1"/>
+    <col min="15" max="15" width="14.77734375" customWidth="1"/>
+    <col min="16" max="16" width="20.21875" customWidth="1"/>
+    <col min="17" max="17" width="30.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B2" s="2"/>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="6"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="O2" s="2"/>
+      <c r="P2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="M2" s="3"/>
+      <c r="Q2" s="6"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="2"/>
+      <c r="G3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="2"/>
+      <c r="J3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="K3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="L3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="M3" s="2"/>
+      <c r="N3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="O3" s="2"/>
+      <c r="P3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="Q3" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B4" s="6" t="s">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B4" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="1">
@@ -574,33 +588,45 @@
       <c r="E4" s="1">
         <v>1.6180000000000001</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="1">
         <v>1.478</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>13.442</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="1">
         <v>1.07</v>
       </c>
-      <c r="I4" s="1">
+      <c r="K4" s="1">
         <v>42.168999999999997</v>
       </c>
-      <c r="J4" s="1">
+      <c r="L4" s="1">
         <v>1.399</v>
       </c>
-      <c r="K4" s="1">
+      <c r="M4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="1">
         <v>962.18399999999997</v>
       </c>
-      <c r="L4" s="1">
+      <c r="O4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="P4" s="1">
         <v>72.5</v>
       </c>
-      <c r="M4" s="1">
+      <c r="Q4" s="1">
         <v>16.59</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B5" s="6" t="s">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="1">
@@ -612,33 +638,45 @@
       <c r="E5" s="1">
         <v>0.42599999999999999</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="1">
         <v>1.468</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>22.475999999999999</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="1">
         <v>0.99099999999999999</v>
       </c>
-      <c r="I5" s="1">
+      <c r="K5" s="1">
         <v>39.646999999999998</v>
       </c>
-      <c r="J5" s="1">
+      <c r="L5" s="1">
         <v>1.2729999999999999</v>
       </c>
-      <c r="K5" s="1">
+      <c r="M5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="1">
         <v>1031.3230000000001</v>
       </c>
-      <c r="L5" s="1">
+      <c r="O5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="P5" s="1">
         <v>69.33</v>
       </c>
-      <c r="M5" s="1">
+      <c r="Q5" s="1">
         <v>13.25</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B6" s="6" t="s">
+    <row r="6" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="1">
@@ -650,33 +688,45 @@
       <c r="E6" s="1">
         <v>0.42799999999999999</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="1">
         <v>1.431</v>
       </c>
-      <c r="G6" s="1">
+      <c r="H6" s="1">
         <v>17.902000000000001</v>
       </c>
-      <c r="H6" s="1">
+      <c r="I6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="1">
         <v>1.1040000000000001</v>
       </c>
-      <c r="I6" s="1">
+      <c r="K6" s="1">
         <v>36.677999999999997</v>
       </c>
-      <c r="J6" s="1">
+      <c r="L6" s="1">
         <v>1.4379999999999999</v>
       </c>
-      <c r="K6" s="1">
+      <c r="M6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="1">
         <v>1046.373</v>
       </c>
-      <c r="L6" s="1">
+      <c r="O6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P6" s="1">
         <v>63.51</v>
       </c>
-      <c r="M6" s="1">
+      <c r="Q6" s="1">
         <v>10.16</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B7" s="6" t="s">
+    <row r="7" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="1">
@@ -687,38 +737,50 @@
         <v>19</v>
       </c>
       <c r="E7" s="1">
-        <f t="shared" ref="D7:M7" si="0">SUM(E4:E6) / 3</f>
+        <f t="shared" ref="E7:Q7" si="0">SUM(E4:E6) / 3</f>
         <v>0.82399999999999995</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="1">
         <f t="shared" si="0"/>
         <v>1.4589999999999999</v>
       </c>
-      <c r="G7" s="1">
+      <c r="H7" s="1">
         <f t="shared" si="0"/>
         <v>17.940000000000001</v>
       </c>
-      <c r="H7" s="1">
+      <c r="I7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="1">
         <f t="shared" si="0"/>
         <v>1.0549999999999999</v>
       </c>
-      <c r="I7" s="1">
-        <f>SUM(I4:I6) / 3</f>
+      <c r="K7" s="1">
+        <f>SUM(K4:K6) / 3</f>
         <v>39.497999999999998</v>
       </c>
-      <c r="J7" s="1">
+      <c r="L7" s="1">
         <f t="shared" si="0"/>
         <v>1.3699999999999999</v>
       </c>
-      <c r="K7" s="1">
+      <c r="M7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="N7" s="1">
         <f t="shared" si="0"/>
         <v>1013.2933333333334</v>
       </c>
-      <c r="L7" s="1">
+      <c r="O7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="P7" s="1">
         <f t="shared" si="0"/>
         <v>68.446666666666658</v>
       </c>
-      <c r="M7" s="1">
+      <c r="Q7" s="1">
         <f t="shared" si="0"/>
         <v>13.333333333333334</v>
       </c>
@@ -726,9 +788,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="C2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="P2:Q2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>